<commit_message>
Reverted back to old modal metadata that works with this version of the modal ui.
</commit_message>
<xml_diff>
--- a/src/rattlesnake/examples/environment/modal/modal_v4.xlsx
+++ b/src/rattlesnake/examples/environment/modal/modal_v4.xlsx
@@ -1,27 +1,213 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmlangs\Desktop\rattlesnake-vibration-controller\src\rattlesnake\examples\environment\modal\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmlangs\Desktop\rattlesnake-vibration-controller-headless\src\rattlesnake\examples\environment\modal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B8CCB0D-929D-4018-A818-A570EAE4B327}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{407E8A28-E39A-4982-84AE-BFD7E0833DF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Modal 0" sheetId="1" r:id="rId1"/>
-    <sheet name="Test Profile" sheetId="2" r:id="rId2"/>
+    <sheet name="Modal 0" sheetId="3" r:id="rId1"/>
+    <sheet name="Test Profile" sheetId="4" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="74">
+  <si>
+    <t>Modal 0</t>
+  </si>
+  <si>
+    <t>Control Type</t>
+  </si>
+  <si>
+    <t>Modal</t>
+  </si>
+  <si>
+    <t>v4.0</t>
+  </si>
+  <si>
+    <t>Samples Per Frame:</t>
+  </si>
+  <si>
+    <t># Number of Samples per Measurement Frame</t>
+  </si>
+  <si>
+    <t>Averaging Type:</t>
+  </si>
+  <si>
+    <t>Linear</t>
+  </si>
+  <si>
+    <t># Averaging Type</t>
+  </si>
+  <si>
+    <t>Number of Averages:</t>
+  </si>
+  <si>
+    <t># Number of Averages used when computing the FRF</t>
+  </si>
+  <si>
+    <t>Averaging Coefficient:</t>
+  </si>
+  <si>
+    <t># Averaging Coefficient for Exponential Averaging</t>
+  </si>
+  <si>
+    <t>FRF Technique:</t>
+  </si>
+  <si>
+    <t>H1</t>
+  </si>
+  <si>
+    <t># FRF Technique</t>
+  </si>
+  <si>
+    <t>FRF Window:</t>
+  </si>
+  <si>
+    <t>rectangle</t>
+  </si>
+  <si>
+    <t># Window used to compute FRF</t>
+  </si>
+  <si>
+    <t>Exponential Window End Value:</t>
+  </si>
+  <si>
+    <t># Exponential Window Value at the end of the measurement frame (0.5 or 50%, not 50)</t>
+  </si>
+  <si>
+    <t>FRF Overlap:</t>
+  </si>
+  <si>
+    <t># Overlap for FRF calculations (0.5 or 50%, not 50)</t>
+  </si>
+  <si>
+    <t>Triggering Type:</t>
+  </si>
+  <si>
+    <t>Free Run</t>
+  </si>
+  <si>
+    <t># One of "Free Run", "First Frame", or "Every Frame"</t>
+  </si>
+  <si>
+    <t>Average Acceptance:</t>
+  </si>
+  <si>
+    <t>Accept All</t>
+  </si>
+  <si>
+    <t># One of "Accept All", "Manual", or "Autoreject"</t>
+  </si>
+  <si>
+    <t>Trigger Channel</t>
+  </si>
+  <si>
+    <t># Channel number (1-based) to use for triggering</t>
+  </si>
+  <si>
+    <t>Pretrigger</t>
+  </si>
+  <si>
+    <t># Amount of frame to use as pretrigger (0.5 or 50%, not 50)</t>
+  </si>
+  <si>
+    <t>Trigger Slope</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t># One of "Positive" or "Negative"</t>
+  </si>
+  <si>
+    <t>Trigger Level</t>
+  </si>
+  <si>
+    <t># Level to use to trigger the test as a fraction of the total range of the channel (0.5 or 50%, not 50)</t>
+  </si>
+  <si>
+    <t>Hysteresis Level</t>
+  </si>
+  <si>
+    <t># Level that a channel must fall below before another trigger can be considered (0.5 or 50%, not 50)</t>
+  </si>
+  <si>
+    <t>Hysteresis Frame Fraction</t>
+  </si>
+  <si>
+    <t># Fraction of the frame that a channel maintain hysteresis condition before another trigger can be considered (0.5 or 50%, not 50)</t>
+  </si>
+  <si>
+    <t>Signal Generator Type</t>
+  </si>
+  <si>
+    <t>random</t>
+  </si>
+  <si>
+    <t># One of "None", "Random", "Burst Random", "Pseudorandom", "Chirp", "Square", or "Sine"</t>
+  </si>
+  <si>
+    <t>Signal Generator Level</t>
+  </si>
+  <si>
+    <t># RMS voltage level for random signals, Peak voltage level for chirp, sine, and square pulse</t>
+  </si>
+  <si>
+    <t>Signal Generator Frequency 1</t>
+  </si>
+  <si>
+    <t># Minimum frequency for broadband signals or frequency for sine and square pulse</t>
+  </si>
+  <si>
+    <t>Signal Generator Frequency 2</t>
+  </si>
+  <si>
+    <t># Maximum frequency for broadband signals.  Ignored for sine and square pulse</t>
+  </si>
+  <si>
+    <t>Signal Generator On Fraction</t>
+  </si>
+  <si>
+    <t># Fraction of time that the burst or square wave is on (0.5 or 50%, not 50)</t>
+  </si>
+  <si>
+    <t>Wait Time for Steady State</t>
+  </si>
+  <si>
+    <t># Time to wait after output starts to allow the system to reach steady state</t>
+  </si>
+  <si>
+    <t>Autoaccept Script</t>
+  </si>
+  <si>
+    <t># File in which an autoacceptance function is defined</t>
+  </si>
+  <si>
+    <t>Autoaccept Function</t>
+  </si>
+  <si>
+    <t># Function name in which the autoacceptance function is defined</t>
+  </si>
+  <si>
+    <t>Reference Channels</t>
+  </si>
+  <si>
+    <t>Disabled Channels</t>
+  </si>
+  <si>
+    <t># List of channels, one per cell on this row</t>
+  </si>
   <si>
     <t>Time (s)</t>
   </si>
@@ -44,12 +230,12 @@
     <t>Start Streaming</t>
   </si>
   <si>
-    <t>Modal 0</t>
-  </si>
-  <si>
     <t>Start Environment</t>
   </si>
   <si>
+    <t>10.0</t>
+  </si>
+  <si>
     <t>Stop Environment</t>
   </si>
   <si>
@@ -57,204 +243,6 @@
   </si>
   <si>
     <t>Stop Hardware</t>
-  </si>
-  <si>
-    <t>Control Type</t>
-  </si>
-  <si>
-    <t>Modal</t>
-  </si>
-  <si>
-    <t>v4.0</t>
-  </si>
-  <si>
-    <t>Samples Per Frame:</t>
-  </si>
-  <si>
-    <t># Number of Samples per Measurement Frame</t>
-  </si>
-  <si>
-    <t>Averaging Type:</t>
-  </si>
-  <si>
-    <t>Linear</t>
-  </si>
-  <si>
-    <t># Averaging Type</t>
-  </si>
-  <si>
-    <t>Number of Averages:</t>
-  </si>
-  <si>
-    <t># Number of Averages used when computing the FRF</t>
-  </si>
-  <si>
-    <t>Averaging Coefficient:</t>
-  </si>
-  <si>
-    <t># Averaging Coefficient for Exponential Averaging</t>
-  </si>
-  <si>
-    <t>FRF Technique:</t>
-  </si>
-  <si>
-    <t>H1</t>
-  </si>
-  <si>
-    <t># FRF Technique</t>
-  </si>
-  <si>
-    <t>FRF Window:</t>
-  </si>
-  <si>
-    <t>rectangle</t>
-  </si>
-  <si>
-    <t># Window used to compute FRF</t>
-  </si>
-  <si>
-    <t>Exponential Window End Value:</t>
-  </si>
-  <si>
-    <t># Exponential Window Value at the end of the measurement frame (0.5 or 50%, not 50)</t>
-  </si>
-  <si>
-    <t>FRF Overlap:</t>
-  </si>
-  <si>
-    <t># Overlap for FRF calculations (0.5 or 50%, not 50)</t>
-  </si>
-  <si>
-    <t>Triggering Type:</t>
-  </si>
-  <si>
-    <t>Free Run</t>
-  </si>
-  <si>
-    <t># One of "Free Run", "First Frame", or "Every Frame"</t>
-  </si>
-  <si>
-    <t>Average Acceptance:</t>
-  </si>
-  <si>
-    <t>Accept All</t>
-  </si>
-  <si>
-    <t># One of "Accept All", "Manual", or "Autoreject"</t>
-  </si>
-  <si>
-    <t>Trigger Channel</t>
-  </si>
-  <si>
-    <t># Channel number (1-based) to use for triggering</t>
-  </si>
-  <si>
-    <t>Pretrigger</t>
-  </si>
-  <si>
-    <t># Amount of frame to use as pretrigger (0.5 or 50%, not 50)</t>
-  </si>
-  <si>
-    <t>Trigger Slope</t>
-  </si>
-  <si>
-    <t>Negative</t>
-  </si>
-  <si>
-    <t># One of "Positive" or "Negative"</t>
-  </si>
-  <si>
-    <t>Trigger Level</t>
-  </si>
-  <si>
-    <t># Level to use to trigger the test as a fraction of the total range of the channel (0.5 or 50%, not 50)</t>
-  </si>
-  <si>
-    <t>Hysteresis Level</t>
-  </si>
-  <si>
-    <t># Level that a channel must fall below before another trigger can be considered (0.5 or 50%, not 50)</t>
-  </si>
-  <si>
-    <t>Hysteresis Frame Fraction</t>
-  </si>
-  <si>
-    <t># Fraction of the frame that a channel maintain hysteresis condition before another trigger can be considered (0.5 or 50%, not 50)</t>
-  </si>
-  <si>
-    <t>Signal Generator Type</t>
-  </si>
-  <si>
-    <t>random</t>
-  </si>
-  <si>
-    <t># One of "None", "Random", "Burst Random", "Pseudorandom", "Chirp", "Square", or "Sine"</t>
-  </si>
-  <si>
-    <t>Signal Generator Level</t>
-  </si>
-  <si>
-    <t># RMS voltage level for random signals, Peak voltage level for chirp, sine, and square pulse</t>
-  </si>
-  <si>
-    <t>Signal Generator Frequency 1</t>
-  </si>
-  <si>
-    <t># Minimum frequency for broadband signals or frequency for sine and square pulse</t>
-  </si>
-  <si>
-    <t>Signal Generator Frequency 2</t>
-  </si>
-  <si>
-    <t># Maximum frequency for broadband signals.  Ignored for sine and square pulse</t>
-  </si>
-  <si>
-    <t>Signal Generator On Fraction</t>
-  </si>
-  <si>
-    <t># Fraction of time that the burst or square wave is on (0.5 or 50%, not 50)</t>
-  </si>
-  <si>
-    <t>Wait Time for Steady State</t>
-  </si>
-  <si>
-    <t># Time to wait after output starts to allow the system to reach steady state</t>
-  </si>
-  <si>
-    <t>Autoaccept Script</t>
-  </si>
-  <si>
-    <t># File in which an autoacceptance function is defined</t>
-  </si>
-  <si>
-    <t>Autoaccept Function</t>
-  </si>
-  <si>
-    <t># Function name in which the autoacceptance function is defined</t>
-  </si>
-  <si>
-    <t>Reference Channels</t>
-  </si>
-  <si>
-    <t>Disabled Channels</t>
-  </si>
-  <si>
-    <t># List of channels, one per cell on this row</t>
-  </si>
-  <si>
-    <t>15.0</t>
-  </si>
-  <si>
-    <t>8.0</t>
-  </si>
-  <si>
-    <t>Change Savefile</t>
-  </si>
-  <si>
-    <t>6.0</t>
-  </si>
-  <si>
-    <t>5.0</t>
   </si>
 </sst>
 </file>
@@ -593,282 +581,282 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D27"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="C1" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="B2">
         <v>1000</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>19</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="B4">
         <v>30</v>
       </c>
       <c r="C4" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0.1</v>
       </c>
       <c r="C5" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="B8">
         <v>0.25</v>
       </c>
       <c r="C8" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="B9">
         <v>0</v>
       </c>
       <c r="C9" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="B10" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="C10" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="C11" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="B12">
         <v>0</v>
       </c>
       <c r="C12" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="B13">
         <v>0</v>
       </c>
       <c r="C13" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="B14" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="C14" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="B15">
         <v>0</v>
       </c>
       <c r="C15" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="B16">
         <v>0</v>
       </c>
       <c r="C16" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="B17">
         <v>0</v>
       </c>
       <c r="C17" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="B18" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="C18" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="B19">
         <v>0.01</v>
       </c>
       <c r="C19" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="B20">
         <v>0</v>
       </c>
       <c r="C20" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="B21">
         <v>500</v>
       </c>
       <c r="C21" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="B22">
         <v>0</v>
       </c>
       <c r="C22" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="B23">
         <v>0</v>
       </c>
       <c r="C23" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="C24" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="C25" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="B26">
         <v>13</v>
@@ -882,10 +870,10 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="C27" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -894,110 +882,77 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D9"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>63</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>64</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>66</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>67</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>66</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C3" t="s">
-        <v>8</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C4" t="s">
-        <v>9</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="B5" t="s">
-        <v>7</v>
+        <v>67</v>
       </c>
       <c r="C5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B6" t="s">
-        <v>7</v>
+        <v>67</v>
       </c>
       <c r="C6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
         <v>73</v>
-      </c>
-      <c r="B7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>73</v>
-      </c>
-      <c r="B8" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>73</v>
-      </c>
-      <c r="B9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C9" t="s">
-        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>